<commit_message>
test: correcoes na suite pytest e geracao de casos de teste
</commit_message>
<xml_diff>
--- a/test_automation/dados/casos_de_teste.xlsx
+++ b/test_automation/dados/casos_de_teste.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Casos de Teste" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Teste'!$A$1:$M$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Teste'!$A$1:$M$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M91"/>
+  <dimension ref="A1:M111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -593,7 +593,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>nome='', email='paciente.b49f22be@teste.cedro', senha='Teste@123', tipoUsuario='paciente'</t>
+          <t>nome='', email='paciente.0e265bea@teste.cedro', senha='Teste@123', tipoUsuario='paciente'</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>nome='Maria Teste', email='paciente.71cfdd6f@teste.cedro', senha='Abc@12', tipoUsuario='paciente'</t>
+          <t>nome='Maria Teste', email='paciente.c6bd08dd@teste.cedro', senha='Abc@12', tipoUsuario='paciente'</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>nome='Maria Teste', email='paciente.278a391b@teste.cedro', senha='Teste@abc', tipoUsuario='paciente'</t>
+          <t>nome='Maria Teste', email='paciente.56ec0385@teste.cedro', senha='Teste@abc', tipoUsuario='paciente'</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>nome='Maria Teste', email='paciente.9ca5ab37@teste.cedro', senha='Teste123', tipoUsuario='paciente'</t>
+          <t>nome='Maria Teste', email='paciente.78e2aefd@teste.cedro', senha='Teste123', tipoUsuario='paciente'</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>nome='Admin Fake', email='adminfake.da32648e@teste.cedro', senha='Teste@123', tipoUsuario='admin'</t>
+          <t>nome='Admin Fake', email='adminfake.d3c64b8d@teste.cedro', senha='Teste@123', tipoUsuario='admin'</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>nome='Dr. João Teste', email='psicologo.365f5588@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/3E0226', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual', precoSessao=150.00</t>
+          <t>nome='Dr. João Teste', email='psicologo.6e922750@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/03EFB9', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual', precoSessao=150.00</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>nome='Dr. João Teste', email='psicologo.c1844e2c@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual', precoSessao=150.00</t>
+          <t>nome='Dr. João Teste', email='psicologo.f04b11e8@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual', precoSessao=150.00</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>nome='Dr. João Teste', email='psicologo.08c030fa@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='12345', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual', precoSessao=150.00</t>
+          <t>nome='Dr. João Teste', email='psicologo.4694a98b@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='12345', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual', precoSessao=150.00</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>nome='Dr. João Teste', email='psicologo.1b9f09b5@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/123456', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual', precoSessao=150.00</t>
+          <t>nome='Dr. João Teste', email='psicologo.d02248ab@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/123456', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual', precoSessao=150.00</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>nome='Dr. João Teste', email='psicologo.4269e128@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/3E0226', tipoPsicologo='Terapia Individual', precoSessao=150.00</t>
+          <t>nome='Dr. João Teste', email='psicologo.42029349@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/03EFB9', tipoPsicologo='Terapia Individual', precoSessao=150.00</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>nome='Dr. João Teste', email='psicologo.afbfec1e@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/3E0226', especialidade='Psicologia Clínica', precoSessao=150.00</t>
+          <t>nome='Dr. João Teste', email='psicologo.3ccb9a73@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/03EFB9', especialidade='Psicologia Clínica', precoSessao=150.00</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>nome='Dr. João Teste', email='psicologo.579851d8@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/3E0226', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual'</t>
+          <t>nome='Dr. João Teste', email='psicologo.e57d2a3b@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/03EFB9', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual'</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>nome='Dr. João Teste', email='psicologo.0dc29a1c@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/3E0226', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual', precoSessao=0</t>
+          <t>nome='Dr. João Teste', email='psicologo.66049189@teste.cedro', senha='Teste@123', tipoUsuario='psicologo', crp='06/03EFB9', especialidade='Psicologia Clínica', tipoPsicologo='Terapia Individual', precoSessao=0</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>email='naoexiste.a45b5ee3@teste.cedro', senha='Cedro@123'</t>
+          <t>email='naoexiste.1d273087@teste.cedro', senha='Cedro@123'</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1565,32 +1565,32 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Agendamento de Sessão</t>
+          <t>Login Social (Google)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Verificar agendamento de sessão com dados válidos</t>
+          <t>Verificar rejeição de login Google com credential vazio</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT). Psicólogo válido com horário livre.</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>psicologoId=&lt;id_psicologo_demo&gt;, dataSessao='2026-08-14T10:00:00', duracao=60, observacoes='Sessão de teste'</t>
+          <t>credential='' (vazio)</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo (POST /api/auth/login). 2. Enviar POST /api/sessoes com header Authorization: Bearer &lt;token&gt;. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar POST /api/auth/google com body {credential: ''}. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>HTTP 201 com a Sessao criada (pacienteId = id do token, valor = precoSessao do psicólogo)</t>
+          <t>HTTP 400 com body {"error": "Token do Google nao fornecido"}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -1600,7 +1600,7 @@
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Campo obrigatório vazio</t>
         </is>
       </c>
     </row>
@@ -1612,32 +1612,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Agendamento de Sessão</t>
+          <t>Login Social (Google)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de agendamento com psicólogo inexistente</t>
+          <t>Verificar rejeição de login Google com token inválido</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>psicologoId=999999, dataSessao='2026-08-14T10:00:00', duracao=60</t>
+          <t>credential='token_invalido_nao_e_jwt'</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes com psicologoId inexistente. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar POST /api/auth/google com credential inválido. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Psicólogo não encontrado"}</t>
+          <t>HTTP 400 (falha na decodificação do JWT do Google — validação manual: issuer, expiração, email_verified)</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -1647,7 +1647,7 @@
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Cenário Negativo</t>
+          <t>Cenário Negativo — token malformado</t>
         </is>
       </c>
     </row>
@@ -1659,32 +1659,32 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Agendamento de Sessão</t>
+          <t>Login Social (Google)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de agendamento com horário ocupado</t>
+          <t>Verificar que login Google cria conta automaticamente para email novo</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado. Já existe sessão não-cancelada do psicólogo no mesmo horário.</t>
+          <t>Email Google não cadastrado no sistema.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>psicologoId=&lt;id_psicologo_demo&gt;, dataSessao='2026-08-14T10:00:00', duracao=60 (mesmo horário de sessão existente)</t>
+          <t>credential=&lt;id_token_google_válido_de_email_novo&gt;</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes com horário já ocupado. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter ID token válido do Google (requer conta Google real). 2. Enviar POST /api/auth/google com o credential. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Horario indisponivel"}</t>
+          <t>HTTP 200 com {token, usuario} — conta criada automaticamente com senha aleatória 'google_oauth_&lt;timestamp&gt;'</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1694,7 +1694,7 @@
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>Registro duplicado — horário do psicólogo</t>
+          <t>Cenário Positivo — requer token Google real (teste manual)</t>
         </is>
       </c>
     </row>
@@ -1711,27 +1711,27 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de agendamento sem psicologoId (campo obrigatório)</t>
+          <t>Verificar agendamento de sessão com dados válidos</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Paciente autenticado (JWT). Psicólogo válido com horário livre.</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>dataSessao='2026-08-14T10:00:00', duracao=60</t>
+          <t>psicologoId=&lt;id_psicologo_demo&gt;, dataSessao='2026-08-21T10:00:00', duracao=60, observacoes='Sessão de teste'</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes sem o campo psicologoId. 3. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo (POST /api/auth/login). 2. Enviar POST /api/sessoes com header Authorization: Bearer &lt;token&gt;. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 (validação @NotNull — 'psicologoId é obrigatório')</t>
+          <t>HTTP 201 com a Sessao criada (pacienteId = id do token, valor = precoSessao do psicólogo)</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1741,7 +1741,7 @@
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Campo obrigatório vazio</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de agendamento sem dataSessao (campo obrigatório)</t>
+          <t>Verificar rejeição de agendamento com psicólogo inexistente</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1768,17 +1768,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>psicologoId=&lt;id_psicologo_demo&gt;, duracao=60</t>
+          <t>psicologoId=999999, dataSessao='2026-08-21T10:00:00', duracao=60</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes sem o campo dataSessao. 3. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes com psicologoId inexistente. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 (validação @NotNull — 'dataSessao é obrigatória')</t>
+          <t>HTTP 400 com body {"error": "Psicólogo não encontrado"}</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -1788,7 +1788,7 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Campo obrigatório vazio</t>
+          <t>Cenário Negativo</t>
         </is>
       </c>
     </row>
@@ -1805,27 +1805,27 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de agendamento sem token JWT (acesso não autorizado)</t>
+          <t>Verificar rejeição de agendamento com horário ocupado</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente autenticado. Já existe sessão não-cancelada do psicólogo no mesmo horário.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>psicologoId=&lt;id_psicologo_demo&gt;, dataSessao='2026-08-14T10:00:00', duracao=60 (sem header Authorization)</t>
+          <t>psicologoId=&lt;id_psicologo_demo&gt;, dataSessao='2026-08-21T10:00:00', duracao=60 (mesmo horário de sessão existente)</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/sessoes sem header Authorization. 2. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes com horário já ocupado. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401 (endpoint exige JWT — SecurityConfig)</t>
+          <t>HTTP 400 com body {"error": "Horario indisponivel"}</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -1835,7 +1835,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Registro duplicado — horário do psicólogo</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Verificar que o backend ignora o pacienteId enviado no body</t>
+          <t>Verificar rejeição de agendamento sem psicologoId (campo obrigatório)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1862,17 +1862,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>pacienteId=999999, psicologoId=&lt;id_psicologo_demo&gt;, dataSessao='2026-08-14T11:00:00', duracao=60</t>
+          <t>dataSessao='2026-08-21T10:00:00', duracao=60</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes com pacienteId diferente do token. 3. Verificar o pacienteId da sessão criada.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes sem o campo psicologoId. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>HTTP 201 — o controller força request.setPacienteId(userId) do token (ignora pacienteId do body)</t>
+          <t>HTTP 400 (validação @NotNull — 'psicologoId é obrigatório')</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -1882,7 +1882,7 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Regra de negócio — segurança</t>
+          <t>Campo obrigatório vazio</t>
         </is>
       </c>
     </row>
@@ -1899,27 +1899,27 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Verificar o limite de 4 sessões gratuitas por mês</t>
+          <t>Verificar rejeição de agendamento sem dataSessao (campo obrigatório)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Paciente não-premium com 4 sessões não-canceladas criadas no mês corrente.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>psicologoId=&lt;id_psicologo_demo&gt;, dataSessao='2026-08-14T14:00:00', duracao=60 (5ª sessão do mês)</t>
+          <t>psicologoId=&lt;id_psicologo_demo&gt;, duracao=60</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo (não-premium). 2. Enviar POST /api/sessoes pela 5ª vez no mês. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes sem o campo dataSessao. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>HTTP 403 com body {"error": "Voce atingiu o limite de 4 sessoes agendadas neste mes no plano gratuito."}</t>
+          <t>HTTP 400 (validação @NotNull — 'dataSessao é obrigatória')</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -1929,7 +1929,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Valor no limite (máx) — 4 sessões/mês para plano gratuito</t>
+          <t>Campo obrigatório vazio</t>
         </is>
       </c>
     </row>
@@ -1941,32 +1941,32 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Pagamento e Confirmação de Sessão</t>
+          <t>Agendamento de Sessão</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Verificar confirmação de pagamento pelo paciente dono da sessão</t>
+          <t>Verificar rejeição de agendamento sem token JWT (acesso não autorizado)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT). Sessão criada com status 'pendente' pertencente ao paciente.</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sessaoId=&lt;id_sessao_do_paciente&gt;</t>
+          <t>psicologoId=&lt;id_psicologo_demo&gt;, dataSessao='2026-08-21T10:00:00', duracao=60 (sem header Authorization)</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes/{id}/confirmar-pagamento com o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar POST /api/sessoes sem header Authorization. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body contendo "message": "Sessão confirmada com sucesso" e a sessão com status 'agendada'</t>
+          <t>HTTP 401 (endpoint exige JWT — SecurityConfig)</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -1976,7 +1976,7 @@
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo — PIX fake do frontend não é testado; apenas o endpoint real de confirmação</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -1988,32 +1988,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Pagamento e Confirmação de Sessão</t>
+          <t>Agendamento de Sessão</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de confirmação de pagamento por outro paciente</t>
+          <t>Verificar que o backend ignora o pacienteId enviado no body</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Paciente A autenticado. Sessão pertencente ao Paciente B.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>sessaoId=&lt;id_sessao_do_paciente_B&gt; (token do paciente A)</t>
+          <t>pacienteId=999999, psicologoId=&lt;id_psicologo_demo&gt;, dataSessao='2026-08-21T11:00:00', duracao=60</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente A. 2. Enviar POST /api/sessoes/{id}/confirmar-pagamento da sessão do paciente B. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes com pacienteId diferente do token. 3. Verificar o pacienteId da sessão criada.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>HTTP 403 com body {"error": "Acesso negado. Paciente não corresponde à sessão."}</t>
+          <t>HTTP 201 — o controller força request.setPacienteId(userId) do token (ignora pacienteId do body)</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -2023,7 +2023,7 @@
       <c r="L33" s="2" t="inlineStr"/>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Regra de negócio — segurança</t>
         </is>
       </c>
     </row>
@@ -2035,32 +2035,32 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Pagamento e Confirmação de Sessão</t>
+          <t>Agendamento de Sessão</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de confirmação de pagamento sem token JWT</t>
+          <t>Verificar o limite de 4 sessões gratuitas por mês</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Sessão existente no sistema.</t>
+          <t>Paciente não-premium com 4 sessões não-canceladas criadas no mês corrente.</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>sessaoId=&lt;id_sessao&gt; (sem header Authorization)</t>
+          <t>psicologoId=&lt;id_psicologo_demo&gt;, dataSessao='2026-08-21T14:00:00', duracao=60 (5ª sessão do mês)</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/sessoes/{id}/confirmar-pagamento sem token. 2. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo (não-premium). 2. Enviar POST /api/sessoes pela 5ª vez no mês. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401 (endpoint exige JWT)</t>
+          <t>HTTP 403 com body {"error": "Voce atingiu o limite de 4 sessoes agendadas neste mes no plano gratuito."}</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -2070,7 +2070,7 @@
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Valor no limite (máx) — 4 sessões/mês para plano gratuito</t>
         </is>
       </c>
     </row>
@@ -2082,32 +2082,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Pagamento e Confirmação de Sessão</t>
+          <t>Sessões</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de confirmação de pagamento de sessão inexistente</t>
+          <t>Verificar listagem das sessões do paciente autenticado</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Paciente autenticado (JWT) com ao menos uma sessão criada.</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>sessaoId=999999</t>
+          <t>Nenhum (GET)</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes/999999/confirmar-pagamento. 3. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar GET /api/sessoes/minhas com o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 (sessão não encontrada — RuntimeException 'Não encontrada' tratada pelo GlobalExceptionHandler)</t>
+          <t>HTTP 200 com lista de sessões onde pacienteId = id do token</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -2117,7 +2117,7 @@
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Cenário Negativo</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -2129,32 +2129,32 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Pagamento e Confirmação de Sessão</t>
+          <t>Sessões</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Verificar o link de reunião antes da janela de liberação (15 min)</t>
+          <t>Verificar listagem de sessões sem token JWT</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado. Sessão confirmada com data futura (mais de 15 min de antecedência).</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>sessaoId=&lt;id_sessao_confirmada&gt;</t>
+          <t>Nenhum (GET, sem token)</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar GET /api/sessoes/{id}/link-reuniao. 3. Verificar o corpo da resposta.</t>
+          <t>1. Enviar GET /api/sessoes/minhas sem header Authorization. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"liberado": false, "disponivelEm": "&lt;ISO datetime&gt;"}</t>
+          <t>HTTP 401 (endpoint exige JWT)</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -2164,7 +2164,7 @@
       <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Valor no limite — janela de liberação de 15 minutos (GOOGLE_MEET_RELEASE_MINUTES_BEFORE)</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -2176,32 +2176,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Pagamento e Confirmação de Sessão</t>
+          <t>Sessões</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Verificar acesso ao link de reunião de outro usuário</t>
+          <t>Verificar cancelamento de sessão pelo paciente dono</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Paciente A autenticado. Sessão pertencente ao Paciente B.</t>
+          <t>Paciente autenticado (JWT). Sessão existente pertencente ao paciente.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>sessaoId=&lt;id_sessao_do_paciente_B&gt; (token do paciente A)</t>
+          <t>sessaoId=&lt;id_sessao_do_paciente&gt;</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente A. 2. Enviar GET /api/sessoes/{id}/link-reuniao da sessão do paciente B. 3. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar DELETE /api/sessoes/{id} com o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>HTTP 403 (apenas admin, paciente ou psicólogo da sessão)</t>
+          <t>HTTP 200 com body {"message": "Deletada"}</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -2211,7 +2211,7 @@
       <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -2223,32 +2223,32 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Chat (Mensagens)</t>
+          <t>Sessões</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Verificar envio de mensagem com dados válidos</t>
+          <t>Verificar rejeição de cancelamento de sessão de outro paciente</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Paciente e psicólogo autenticados (JWTs).</t>
+          <t>Paciente A autenticado. Sessão pertencente ao Paciente B.</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>destinatarioId=&lt;id_psicologo_demo&gt;, mensagem='Olá, gostaria de agendar uma sessão'</t>
+          <t>sessaoId=&lt;id_sessao_paciente_B&gt; (token do paciente A)</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/mensagens com header Authorization: Bearer &lt;token&gt;. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente A. 2. Enviar DELETE /api/sessoes/{id} da sessão do paciente B. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com a Mensagem criada (remetenteId = id do token)</t>
+          <t>HTTP 403 (apenas o paciente dono ou admin pode cancelar)</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -2258,7 +2258,7 @@
       <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -2270,32 +2270,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Chat (Mensagens)</t>
+          <t>Sessões</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de mensagem com mais de 2000 caracteres</t>
+          <t>Verificar consulta de disponibilidade de horários do psicólogo</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Sistema no ar. Psicólogo demo cadastrado.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>destinatarioId=&lt;id_psicologo_demo&gt;, mensagem='&lt;2001 caracteres&gt;'</t>
+          <t>psicologoId=&lt;id_psicologo_demo&gt;, data='2026-08-21'</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/mensagens com mensagem de 2001 caracteres. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar GET /api/sessoes/disponibilidade/{{psicologoId}}?data={data_futura}. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Mensagem muito longa (máx. 2000 caracteres)"}</t>
+          <t>HTTP 200 com body {data, horariosDisponiveis: [...], horariosOcupados: [...]} — horários base: 08:00, 09:00, 10:00, 11:00, 14:00, 15:00, 16:00, 17:00, 18:00</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -2305,7 +2305,7 @@
       <c r="L39" s="2" t="inlineStr"/>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>Valor no limite (máx) — 2000 caracteres</t>
+          <t>Cenário Positivo — endpoint público</t>
         </is>
       </c>
     </row>
@@ -2317,32 +2317,32 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Chat (Mensagens)</t>
+          <t>Sessões</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Verificar envio de mensagem com exatamente 2000 caracteres (limite)</t>
+          <t>Verificar disponibilidade de psicólogo inexistente</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>destinatarioId=&lt;id_psicologo_demo&gt;, mensagem='&lt;2000 caracteres&gt;'</t>
+          <t>psicologoId=999999, data='2026-08-21'</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/mensagens com mensagem de exatamente 2000 caracteres. 3. Verificar o código HTTP.</t>
+          <t>1. Enviar GET /api/sessoes/disponibilidade/999999?data={data_futura}. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 — mensagem aceita no limite máximo</t>
+          <t>HTTP 400 (psicólogo não encontrado)</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -2352,7 +2352,7 @@
       <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>Valor no limite (máx)</t>
+          <t>Cenário Negativo</t>
         </is>
       </c>
     </row>
@@ -2364,32 +2364,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Chat (Mensagens)</t>
+          <t>Pagamento e Confirmação de Sessão</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de mensagem sem destinatarioId (campo obrigatório)</t>
+          <t>Verificar confirmação de pagamento pelo paciente dono da sessão</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Paciente autenticado (JWT). Sessão criada com status 'pendente' pertencente ao paciente.</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>mensagem='Olá' (sem destinatarioId)</t>
+          <t>sessaoId=&lt;id_sessao_do_paciente&gt;</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/mensagens sem o campo destinatarioId. 3. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes/{id}/confirmar-pagamento com o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 (validação @NotNull do campo destinatarioId)</t>
+          <t>HTTP 200 com body contendo "message": "Sessão confirmada com sucesso" e a sessão com status 'agendada'</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -2399,7 +2399,7 @@
       <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>Campo obrigatório vazio</t>
+          <t>Cenário Positivo — PIX fake do frontend não é testado; apenas o endpoint real de confirmação</t>
         </is>
       </c>
     </row>
@@ -2411,32 +2411,32 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Chat (Mensagens)</t>
+          <t>Pagamento e Confirmação de Sessão</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de mensagem sem token JWT</t>
+          <t>Verificar rejeição de confirmação de pagamento por outro paciente</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente A autenticado. Sessão pertencente ao Paciente B.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>destinatarioId=&lt;id_psicologo_demo&gt;, mensagem='Olá' (sem token)</t>
+          <t>sessaoId=&lt;id_sessao_do_paciente_B&gt; (token do paciente A)</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/mensagens sem header Authorization. 2. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente A. 2. Enviar POST /api/sessoes/{id}/confirmar-pagamento da sessão do paciente B. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401 (endpoint exige JWT)</t>
+          <t>HTTP 403 com body {"error": "Acesso negado. Paciente não corresponde à sessão."}</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -2458,32 +2458,32 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Chat (Mensagens)</t>
+          <t>Pagamento e Confirmação de Sessão</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Verificar que apenas o destinatário pode marcar mensagem como lida</t>
+          <t>Verificar rejeição de confirmação de pagamento sem token JWT</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Mensagem existente entre paciente e psicólogo.</t>
+          <t>Sessão existente no sistema.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>mensagemId=&lt;id_mensagem&gt; (token do remetente, não do destinatário)</t>
+          <t>sessaoId=&lt;id_sessao&gt; (sem header Authorization)</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do remetente da mensagem. 2. Enviar PUT /api/mensagens/{id}/lida com o token do remetente. 3. Verificar o código HTTP.</t>
+          <t>1. Enviar POST /api/sessoes/{id}/confirmar-pagamento sem token. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>HTTP 403 (apenas o destinatário pode marcar como lida)</t>
+          <t>HTTP 401 (endpoint exige JWT)</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -2505,32 +2505,32 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Chat (Mensagens)</t>
+          <t>Pagamento e Confirmação de Sessão</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Verificar listagem de conversas do usuário autenticado</t>
+          <t>Verificar rejeição de confirmação de pagamento de sessão inexistente</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado com mensagens trocadas.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Nenhum (GET)</t>
+          <t>sessaoId=999999</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar GET /api/mensagens/conversas com o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/sessoes/999999/confirmar-pagamento. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com lista de ConversaResumo {userId, nome, fotoUrl, ultimaMensagem, dataUltimaMensagem, naoLidas, mensagemEnviada}</t>
+          <t>HTTP 400 (sessão não encontrada — RuntimeException 'Não encontrada' tratada pelo GlobalExceptionHandler)</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -2540,7 +2540,7 @@
       <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Cenário Negativo</t>
         </is>
       </c>
     </row>
@@ -2552,32 +2552,32 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Verificação de CRP</t>
+          <t>Pagamento e Confirmação de Sessão</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Verificar CRP disponível para cadastro</t>
+          <t>Verificar o link de reunião antes da janela de liberação (15 min)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar. CRP não cadastrado.</t>
+          <t>Paciente autenticado. Sessão confirmada com data futura (mais de 15 min de antecedência).</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>crp='06/7336DD'</t>
+          <t>sessaoId=&lt;id_sessao_confirmada&gt;</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/psicologos/verificar-crp?crp=&lt;crp&gt;. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar GET /api/sessoes/{id}/link-reuniao. 3. Verificar o corpo da resposta.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"valido": true, "mensagem": "CRP disponível para cadastro"}</t>
+          <t>HTTP 200 com body {"liberado": false, "disponivelEm": "&lt;ISO datetime&gt;"}</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -2587,7 +2587,7 @@
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Valor no limite — janela de liberação de 15 minutos (GOOGLE_MEET_RELEASE_MINUTES_BEFORE)</t>
         </is>
       </c>
     </row>
@@ -2599,32 +2599,32 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Verificação de CRP</t>
+          <t>Pagamento e Confirmação de Sessão</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de CRP em formato inválido</t>
+          <t>Verificar acesso ao link de reunião de outro usuário</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente A autenticado. Sessão pertencente ao Paciente B.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>crp='12345'</t>
+          <t>sessaoId=&lt;id_sessao_do_paciente_B&gt; (token do paciente A)</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/psicologos/verificar-crp?crp=12345. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente A. 2. Enviar GET /api/sessoes/{id}/link-reuniao da sessão do paciente B. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"valido": false, "mensagem": "Formato de CRP inválido. Use: XX/XXXXXX"}</t>
+          <t>HTTP 403 (apenas admin, paciente ou psicólogo da sessão)</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -2634,7 +2634,7 @@
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Cenário Negativo — formato inválido</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -2646,32 +2646,32 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Verificação de CRP</t>
+          <t>Chat (Mensagens)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de CRP já cadastrado</t>
+          <t>Verificar envio de mensagem com dados válidos</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>CRP 06/123456 já cadastrado (psicólogo demo do seeder).</t>
+          <t>Paciente e psicólogo autenticados (JWTs).</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>crp='06/123456'</t>
+          <t>destinatarioId=&lt;id_psicologo_demo&gt;, mensagem='Olá, gostaria de agendar uma sessão'</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/psicologos/verificar-crp?crp=06/123456. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/mensagens com header Authorization: Bearer &lt;token&gt;. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>HTTP 409 com body {"valido": false, "mensagem": "Este CRP já está cadastrado na plataforma."}</t>
+          <t>HTTP 200 com a Mensagem criada (remetenteId = id do token)</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -2681,7 +2681,7 @@
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Registro duplicado</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -2693,32 +2693,32 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Verificação de CRP</t>
+          <t>Chat (Mensagens)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Verificar CRP com formato no limite (5 dígitos após a barra)</t>
+          <t>Verificar rejeição de mensagem com mais de 2000 caracteres</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>crp='06/4E06E'</t>
+          <t>destinatarioId=&lt;id_psicologo_demo&gt;, mensagem='&lt;2001 caracteres&gt;'</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/psicologos/verificar-crp com CRP de 5 dígitos. 2. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/mensagens com mensagem de 2001 caracteres. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 (formato \d{2}/\d{5,6} aceita 5 ou 6 dígitos) ou HTTP 409 se já cadastrado</t>
+          <t>HTTP 400 com body {"error": "Mensagem muito longa (máx. 2000 caracteres)"}</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -2728,7 +2728,7 @@
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Valor no limite (mín) — 5 dígitos</t>
+          <t>Valor no limite (máx) — 2000 caracteres</t>
         </is>
       </c>
     </row>
@@ -2740,32 +2740,32 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Verificação de CRP</t>
+          <t>Chat (Mensagens)</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Verificar CRP com formato no limite (6 dígitos após a barra)</t>
+          <t>Verificar envio de mensagem com exatamente 2000 caracteres (limite)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>crp='06/7BEE3F'</t>
+          <t>destinatarioId=&lt;id_psicologo_demo&gt;, mensagem='&lt;2000 caracteres&gt;'</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/psicologos/verificar-crp com CRP de 6 dígitos. 2. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/mensagens com mensagem de exatamente 2000 caracteres. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 (formato \d{2}/\d{5,6} aceita 5 ou 6 dígitos) ou HTTP 409 se já cadastrado</t>
+          <t>HTTP 200 — mensagem aceita no limite máximo</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -2775,7 +2775,7 @@
       <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>Valor no limite (máx) — 6 dígitos</t>
+          <t>Valor no limite (máx)</t>
         </is>
       </c>
     </row>
@@ -2787,32 +2787,32 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Verificação de CRP</t>
+          <t>Chat (Mensagens)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Verificar CRP com 7 dígitos (acima do limite)</t>
+          <t>Verificar rejeição de mensagem sem destinatarioId (campo obrigatório)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>crp='06/1234567'</t>
+          <t>mensagem='Olá' (sem destinatarioId)</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/psicologos/verificar-crp?crp=06/1234567. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/mensagens sem o campo destinatarioId. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"valido": false, "mensagem": "Formato de CRP inválido. Use: XX/XXXXXX"}</t>
+          <t>HTTP 400 (validação @NotNull do campo destinatarioId)</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -2822,7 +2822,7 @@
       <c r="L50" s="2" t="inlineStr"/>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>Valor no limite (máx+1) — 7 dígitos é inválido</t>
+          <t>Campo obrigatório vazio</t>
         </is>
       </c>
     </row>
@@ -2834,32 +2834,32 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Alteração de Senha</t>
+          <t>Chat (Mensagens)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Verificar alteração de senha com dados válidos</t>
+          <t>Verificar rejeição de mensagem sem token JWT</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>senhaAtual='Cedro@123', novaSenha='NovaSenha@123'</t>
+          <t>destinatarioId=&lt;id_psicologo_demo&gt;, mensagem='Olá' (sem token)</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/alterar-senha com o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar POST /api/mensagens sem header Authorization. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"message": "Senha alterada"}</t>
+          <t>HTTP 401 (endpoint exige JWT)</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -2869,7 +2869,7 @@
       <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -2881,32 +2881,32 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Alteração de Senha</t>
+          <t>Chat (Mensagens)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de alteração com senha atual incorreta</t>
+          <t>Verificar que apenas o destinatário pode marcar mensagem como lida</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Mensagem existente entre paciente e psicólogo.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>senhaAtual='SenhaErrada@1', novaSenha='NovaSenha@123'</t>
+          <t>mensagemId=&lt;id_mensagem&gt; (token do remetente, não do destinatário)</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/alterar-senha com senha atual errada. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do remetente da mensagem. 2. Enviar PUT /api/mensagens/{id}/lida com o token do remetente. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Senha atual ta errada"}</t>
+          <t>HTTP 403 (apenas o destinatário pode marcar como lida)</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -2916,7 +2916,7 @@
       <c r="L52" s="2" t="inlineStr"/>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>Cenário Negativo</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -2928,32 +2928,32 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Alteração de Senha</t>
+          <t>Chat (Mensagens)</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de nova senha sem número</t>
+          <t>Verificar listagem de conversas do usuário autenticado</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Paciente autenticado com mensagens trocadas.</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>senhaAtual='Cedro@123', novaSenha='NovaSenha@abc'</t>
+          <t>Nenhum (GET)</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/alterar-senha com nova senha sem número. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar GET /api/mensagens/conversas com o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Precisa ter pelo menos 1 numero"}</t>
+          <t>HTTP 200 com lista de ConversaResumo {userId, nome, fotoUrl, ultimaMensagem, dataUltimaMensagem, naoLidas, mensagemEnviada}</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -2963,7 +2963,7 @@
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>Cenário Negativo — validação de força da senha</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -2975,32 +2975,32 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Alteração de Senha</t>
+          <t>Verificação de CRP</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de nova senha sem caractere especial</t>
+          <t>Verificar CRP disponível para cadastro</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Sistema no ar. CRP não cadastrado.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>senhaAtual='Cedro@123', novaSenha='NovaSenha123'</t>
+          <t>crp='06/CA356B'</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/alterar-senha com nova senha sem especial. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar GET /api/psicologos/verificar-crp?crp=&lt;crp&gt;. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Precisa ter pelo menos 1 caractere especial"}</t>
+          <t>HTTP 200 com body {"valido": true, "mensagem": "CRP disponível para cadastro"}</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -3010,7 +3010,7 @@
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Cenário Negativo — validação de força da senha</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -3022,32 +3022,32 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Alteração de Senha</t>
+          <t>Verificação de CRP</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de nova senha com menos de 6 caracteres</t>
+          <t>Verificar rejeição de CRP em formato inválido</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>senhaAtual='Cedro@123', novaSenha='Ab@12'</t>
+          <t>crp='12345'</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/alterar-senha com nova senha de 5 caracteres. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar GET /api/psicologos/verificar-crp?crp=12345. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Senha muito curta (min. 6 caracteres)"}</t>
+          <t>HTTP 400 com body {"valido": false, "mensagem": "Formato de CRP inválido. Use: XX/XXXXXX"}</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -3057,7 +3057,7 @@
       <c r="L55" s="2" t="inlineStr"/>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Valor no limite (mín-1) — 5 caracteres</t>
+          <t>Cenário Negativo — formato inválido</t>
         </is>
       </c>
     </row>
@@ -3069,32 +3069,32 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Alteração de Senha</t>
+          <t>Verificação de CRP</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de alteração de senha sem token JWT</t>
+          <t>Verificar rejeição de CRP já cadastrado</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>CRP 06/123456 já cadastrado (psicólogo demo do seeder).</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>senhaAtual='Cedro@123', novaSenha='NovaSenha@123' (sem token)</t>
+          <t>crp='06/123456'</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar PUT /api/auth/alterar-senha sem header Authorization. 2. Verificar o código HTTP.</t>
+          <t>1. Enviar GET /api/psicologos/verificar-crp?crp=06/123456. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401 (endpoint exige JWT)</t>
+          <t>HTTP 409 com body {"valido": false, "mensagem": "Este CRP já está cadastrado na plataforma."}</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -3104,7 +3104,7 @@
       <c r="L56" s="2" t="inlineStr"/>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Registro duplicado</t>
         </is>
       </c>
     </row>
@@ -3116,32 +3116,32 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Upload de Foto de Perfil</t>
+          <t>Verificação de CRP</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Verificar upload de imagem JPG válida</t>
+          <t>Verificar CRP com formato no limite (5 dígitos após a barra)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT). Arquivo JPG válido de até 2MB.</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>file=&lt;foto.jpg&gt; (multipart/form-data, &lt; 2MB, content-type image/jpeg)</t>
+          <t>crp='06/E063C'</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/auth/foto-perfil-upload com o arquivo e o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar GET /api/psicologos/verificar-crp com CRP de 5 dígitos. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"message": "Foto atualizada", "fotoUrl": "&lt;url&gt;"}</t>
+          <t>HTTP 200 (formato \d{2}/\d{5,6} aceita 5 ou 6 dígitos) ou HTTP 409 se já cadastrado</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -3151,7 +3151,7 @@
       <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Valor no limite (mín) — 5 dígitos</t>
         </is>
       </c>
     </row>
@@ -3163,32 +3163,32 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Upload de Foto de Perfil</t>
+          <t>Verificação de CRP</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de upload de imagem maior que 2MB</t>
+          <t>Verificar CRP com formato no limite (6 dígitos após a barra)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT). Arquivo JPG de 2.1MB.</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>file=&lt;foto_grande.jpg&gt; (multipart/form-data, &gt; 2MB)</t>
+          <t>crp='06/2421BE'</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/auth/foto-perfil-upload com arquivo &gt; 2MB. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar GET /api/psicologos/verificar-crp com CRP de 6 dígitos. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Imagem muito grande (max. 2MB)"}</t>
+          <t>HTTP 200 (formato \d{2}/\d{5,6} aceita 5 ou 6 dígitos) ou HTTP 409 se já cadastrado</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -3198,7 +3198,7 @@
       <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>Valor no limite (máx) — 2MB (2_000_000 bytes)</t>
+          <t>Valor no limite (máx) — 6 dígitos</t>
         </is>
       </c>
     </row>
@@ -3210,32 +3210,32 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Upload de Foto de Perfil</t>
+          <t>Verificação de CRP</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de upload de arquivo sem imagem</t>
+          <t>Verificar CRP com 7 dígitos (acima do limite)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>file=&lt;arquivo.txt&gt; (content-type text/plain)</t>
+          <t>crp='06/1234567'</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/auth/foto-perfil-upload com arquivo .txt. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar GET /api/psicologos/verificar-crp?crp=06/1234567. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Formato invalido. Use JPG, PNG ou WebP"}</t>
+          <t>HTTP 400 com body {"valido": false, "mensagem": "Formato de CRP inválido. Use: XX/XXXXXX"}</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -3245,7 +3245,7 @@
       <c r="L59" s="2" t="inlineStr"/>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>Cenário Negativo — formato inválido</t>
+          <t>Valor no limite (máx+1) — 7 dígitos é inválido</t>
         </is>
       </c>
     </row>
@@ -3257,12 +3257,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Upload de Foto de Perfil</t>
+          <t>Alteração de Senha</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de upload sem arquivo</t>
+          <t>Verificar alteração de senha com dados válidos</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -3272,17 +3272,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>file=&lt;vazio&gt; (multipart/form-data sem arquivo)</t>
+          <t>senhaAtual='Cedro@123', novaSenha='NovaSenha@123'</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/auth/foto-perfil-upload sem arquivo. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/alterar-senha com o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Arquivo de imagem obrigatorio"}</t>
+          <t>HTTP 200 com body {"message": "Senha alterada"}</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -3292,7 +3292,7 @@
       <c r="L60" s="2" t="inlineStr"/>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>Campo obrigatório vazio</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -3304,32 +3304,32 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Upload de Foto de Perfil</t>
+          <t>Alteração de Senha</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de upload sem token JWT</t>
+          <t>Verificar rejeição de alteração com senha atual incorreta</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>file=&lt;foto.jpg&gt; (sem header Authorization)</t>
+          <t>senhaAtual='SenhaErrada@1', novaSenha='NovaSenha@123'</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/auth/foto-perfil-upload sem token. 2. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/alterar-senha com senha atual errada. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401 (endpoint exige JWT)</t>
+          <t>HTTP 400 com body {"error": "Senha atual ta errada"}</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr"/>
@@ -3339,7 +3339,7 @@
       <c r="L61" s="2" t="inlineStr"/>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Cenário Negativo</t>
         </is>
       </c>
     </row>
@@ -3351,32 +3351,32 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Upload de Foto de Perfil</t>
+          <t>Alteração de Senha</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Verificar upload de imagem PNG válida</t>
+          <t>Verificar rejeição de nova senha sem número</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT). Arquivo PNG válido de até 2MB.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>file=&lt;foto.png&gt; (multipart/form-data, &lt; 2MB, content-type image/png)</t>
+          <t>senhaAtual='Cedro@123', novaSenha='NovaSenha@abc'</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/auth/foto-perfil-upload com arquivo PNG. 3. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/alterar-senha com nova senha sem número. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"message": "Foto atualizada", "fotoUrl": "&lt;url&gt;"}</t>
+          <t>HTTP 400 com body {"error": "Precisa ter pelo menos 1 numero"}</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
       <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo — formatos aceitos: JPG, PNG, WebP</t>
+          <t>Cenário Negativo — validação de força da senha</t>
         </is>
       </c>
     </row>
@@ -3398,32 +3398,32 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Assinatura Premium (RevenueCat)</t>
+          <t>Alteração de Senha</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Verificar processamento de webhook autorizado</t>
+          <t>Verificar rejeição de nova senha sem caractere especial</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>REVENUECAT_WEBHOOK_SECRET configurado no backend.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization=&lt;secret&gt;. Body: {"event": {"type": "INITIAL_PURCHASE", "app_user_id": "&lt;id_usuario&gt;", "expiration_at_ms": 1750000000000, "product_id": "premium_mensal", "transaction_id": "tx123"}}</t>
+          <t>senhaAtual='Cedro@123', novaSenha='NovaSenha123'</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/assinatura/webhook com header Authorization correto. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/alterar-senha com nova senha sem especial. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"message": "Webhook processado"}</t>
+          <t>HTTP 400 com body {"error": "Precisa ter pelo menos 1 caractere especial"}</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -3433,7 +3433,7 @@
       <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Cenário Negativo — validação de força da senha</t>
         </is>
       </c>
     </row>
@@ -3445,32 +3445,32 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Assinatura Premium (RevenueCat)</t>
+          <t>Alteração de Senha</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de webhook não autorizado</t>
+          <t>Verificar rejeição de nova senha com menos de 6 caracteres</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization=&lt;secret_errado&gt;</t>
+          <t>senhaAtual='Cedro@123', novaSenha='Ab@12'</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/assinatura/webhook com header Authorization incorreto. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/alterar-senha com nova senha de 5 caracteres. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401 com body {"error": "Webhook nao autorizado"}</t>
+          <t>HTTP 400 com body {"error": "Senha muito curta (min. 6 caracteres)"}</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -3480,7 +3480,7 @@
       <c r="L64" s="2" t="inlineStr"/>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Valor no limite (mín-1) — 5 caracteres</t>
         </is>
       </c>
     </row>
@@ -3492,32 +3492,32 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Assinatura Premium (RevenueCat)</t>
+          <t>Alteração de Senha</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de webhook com payload inválido</t>
+          <t>Verificar rejeição de alteração de senha sem token JWT</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>REVENUECAT_WEBHOOK_SECRET configurado no backend.</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization=&lt;secret&gt;. Body: {"event": {}}</t>
+          <t>senhaAtual='Cedro@123', novaSenha='NovaSenha@123' (sem token)</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/assinatura/webhook com payload sem type/app_user_id. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar PUT /api/auth/alterar-senha sem header Authorization. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Payload RevenueCat invalido"}</t>
+          <t>HTTP 401 (endpoint exige JWT)</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
@@ -3527,7 +3527,7 @@
       <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>Campo obrigatório vazio</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -3539,32 +3539,32 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Assinatura Premium (RevenueCat)</t>
+          <t>Perfil e Conta</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Verificar status de assinatura de usuário free</t>
+          <t>Verificar atualização de perfil com dados válidos</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado sem assinatura ativa.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Nenhum (GET)</t>
+          <t>nome='Novo Nome', telefone='(11) 98888-7777', bio='Minha bio'</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo (não-premium). 2. Enviar GET /api/assinatura/status com o token. 3. Verificar o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/auth/perfil com body {nome, telefone, bio}. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"isPremium": false, "chamadasRealizadas": &lt;count&gt;, "limiteMensal": 4}</t>
+          <t>HTTP 200 com body {"message": "Perfil atualizado"}</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -3574,7 +3574,7 @@
       <c r="L66" s="2" t="inlineStr"/>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo — limite gratuito de 4 sessões/mês</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -3586,12 +3586,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Assinatura Premium (RevenueCat)</t>
+          <t>Perfil e Conta</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Verificar status de assinatura sem token JWT</t>
+          <t>Verificar rejeição de atualização de perfil sem token JWT</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3601,12 +3601,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Nenhum (GET, sem token)</t>
+          <t>nome='Novo Nome' (sem token)</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/assinatura/status sem header Authorization. 2. Verificar o código HTTP.</t>
+          <t>1. Enviar PUT /api/auth/perfil sem header Authorization. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -3633,32 +3633,32 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Gestão de Usuários (Admin)</t>
+          <t>Perfil e Conta</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Verificar listagem de todos os usuários por admin</t>
+          <t>Verificar exclusão de conta pelo próprio usuário</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Admin autenticado (JWT).</t>
+          <t>Usuário de teste autenticado (JWT). Conta criada exclusivamente para este teste.</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Nenhum (GET)</t>
+          <t>Nenhum (DELETE)</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do admin (admin@cedro.com). 2. Enviar GET /api/usuarios com o token. 3. Verificar o código HTTP.</t>
+          <t>1. Criar usuário de teste via POST /api/auth/register. 2. Obter token JWT do usuário de teste. 3. Enviar DELETE /api/auth/conta com o token. 4. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com lista de todos os usuários</t>
+          <t>HTTP 200 com body {"message": "Conta excluída"} — sessões e mensagens relacionadas são deletadas (transacional)</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -3668,7 +3668,7 @@
       <c r="L68" s="2" t="inlineStr"/>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo — NOTA: endpoint expõe senhaHash (vulnerabilidade conhecida)</t>
+          <t>Cenário Positivo — operação destrutiva e irreversível</t>
         </is>
       </c>
     </row>
@@ -3680,32 +3680,32 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Gestão de Usuários (Admin)</t>
+          <t>Perfil e Conta</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de listagem de usuários por não-admin</t>
+          <t>Verificar rejeição de exclusão de conta sem token JWT</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Nenhum (GET, token de paciente)</t>
+          <t>Nenhum (DELETE, sem token)</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar GET /api/usuarios com o token do paciente. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar DELETE /api/auth/conta sem header Authorization. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>HTTP 403 com body {"error": "Acesso negado"}</t>
+          <t>HTTP 401 (endpoint exige JWT)</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -3727,32 +3727,32 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Gestão de Usuários (Admin)</t>
+          <t>Upload de Foto de Perfil</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Verificar que usuário comum só pode ver a si mesmo</t>
+          <t>Verificar upload de imagem JPG válida</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT).</t>
+          <t>Paciente autenticado (JWT). Arquivo JPG válido de até 2MB.</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>id=&lt;id_de_outro_usuario&gt; (token do paciente)</t>
+          <t>file=&lt;foto.jpg&gt; (multipart/form-data, &lt; 2MB, content-type image/jpeg)</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar GET /api/usuarios/{id} de outro usuário. 3. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/auth/foto-perfil-upload com o arquivo e o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>HTTP 403 (se não admin e id não corresponde)</t>
+          <t>HTTP 200 com body {"message": "Foto atualizada", "fotoUrl": "&lt;url&gt;"}</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -3762,7 +3762,7 @@
       <c r="L70" s="2" t="inlineStr"/>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -3774,32 +3774,32 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Gestão de Usuários (Admin)</t>
+          <t>Upload de Foto de Perfil</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Verificar ativação/desativação de usuário por admin</t>
+          <t>Verificar rejeição de upload de imagem maior que 2MB</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Admin autenticado (JWT).</t>
+          <t>Paciente autenticado (JWT). Arquivo JPG de 2.1MB.</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>id=&lt;id_usuario&gt;, body={"ativo": false}</t>
+          <t>file=&lt;foto_grande.jpg&gt; (multipart/form-data, &gt; 2MB)</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do admin. 2. Enviar PUT /api/usuarios/{id}/ativar com ativo=false. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/auth/foto-perfil-upload com arquivo &gt; 2MB. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"message": "ok"}</t>
+          <t>HTTP 400 com body {"error": "Imagem muito grande (max. 2MB)"}</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -3809,7 +3809,7 @@
       <c r="L71" s="2" t="inlineStr"/>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Valor no limite (máx) — 2MB (2_000_000 bytes)</t>
         </is>
       </c>
     </row>
@@ -3821,12 +3821,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Gestão de Usuários (Admin)</t>
+          <t>Upload de Foto de Perfil</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de desativação de usuário por não-admin</t>
+          <t>Verificar rejeição de upload de arquivo sem imagem</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3836,17 +3836,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>id=&lt;id_usuario&gt;, body={"ativo": false} (token de paciente)</t>
+          <t>file=&lt;arquivo.txt&gt; (content-type text/plain)</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/usuarios/{id}/ativar com o token do paciente. 3. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/auth/foto-perfil-upload com arquivo .txt. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>HTTP 403 (apenas admin)</t>
+          <t>HTTP 400 com body {"error": "Formato invalido. Use JPG, PNG ou WebP"}</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -3856,7 +3856,7 @@
       <c r="L72" s="2" t="inlineStr"/>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Cenário Negativo — formato inválido</t>
         </is>
       </c>
     </row>
@@ -3868,32 +3868,32 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Gestão de Usuários (Admin)</t>
+          <t>Upload de Foto de Perfil</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Verificar exclusão de usuário por admin</t>
+          <t>Verificar rejeição de upload sem arquivo</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Admin autenticado (JWT). Usuário de teste criado.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>id=&lt;id_usuario_teste&gt;</t>
+          <t>file=&lt;vazio&gt; (multipart/form-data sem arquivo)</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do admin. 2. Enviar DELETE /api/usuarios/{id} do usuário de teste. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/auth/foto-perfil-upload sem arquivo. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"message": "Deletada"}</t>
+          <t>HTTP 400 com body {"error": "Arquivo de imagem obrigatorio"}</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -3903,7 +3903,7 @@
       <c r="L73" s="2" t="inlineStr"/>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Campo obrigatório vazio</t>
         </is>
       </c>
     </row>
@@ -3915,32 +3915,32 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Lista e Detalhe de Psicólogos</t>
+          <t>Upload de Foto de Perfil</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Verificar listagem pública de psicólogos</t>
+          <t>Verificar rejeição de upload sem token JWT</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar. Psicólogos cadastrados.</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Nenhum (GET, público)</t>
+          <t>file=&lt;foto.jpg&gt; (sem header Authorization)</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/psicologos sem autenticação. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar POST /api/auth/foto-perfil-upload sem token. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com lista de DTOs públicos {id, nome, especialidade, tipoPsicologo, bio, precoSessao, avaliacao, fotoUrl} — sem email, telefone ou senha</t>
+          <t>HTTP 401 (endpoint exige JWT)</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -3950,7 +3950,7 @@
       <c r="L74" s="2" t="inlineStr"/>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -3962,32 +3962,32 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Lista e Detalhe de Psicólogos</t>
+          <t>Upload de Foto de Perfil</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Verificar detalhe de psicólogo inexistente</t>
+          <t>Verificar upload de imagem PNG válida</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente autenticado (JWT). Arquivo PNG válido de até 2MB.</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>id=999999</t>
+          <t>file=&lt;foto.png&gt; (multipart/form-data, &lt; 2MB, content-type image/png)</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/psicologos/999999. 2. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/auth/foto-perfil-upload com arquivo PNG. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 (RuntimeException 'Não encontrado' tratada pelo GlobalExceptionHandler)</t>
+          <t>HTTP 200 com body {"message": "Foto atualizada", "fotoUrl": "&lt;url&gt;"}</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -3997,7 +3997,7 @@
       <c r="L75" s="2" t="inlineStr"/>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>Cenário Negativo</t>
+          <t>Cenário Positivo — formatos aceitos: JPG, PNG, WebP</t>
         </is>
       </c>
     </row>
@@ -4009,32 +4009,32 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Lista e Detalhe de Psicólogos</t>
+          <t>Assinatura Premium (RevenueCat)</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Verificar detalhe de usuário que não é psicólogo</t>
+          <t>Verificar processamento de webhook autorizado</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar. Paciente demo cadastrado.</t>
+          <t>REVENUECAT_WEBHOOK_SECRET configurado no backend.</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>id=&lt;id_paciente_demo&gt;</t>
+          <t>Header Authorization=&lt;secret&gt;. Body: {"event": {"type": "INITIAL_PURCHASE", "app_user_id": "&lt;id_usuario&gt;", "expiration_at_ms": 1750000000000, "product_id": "premium_mensal", "transaction_id": "tx123"}}</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/psicologos/{id} do paciente demo. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar POST /api/assinatura/webhook com header Authorization correto. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Não é psicólogo"}</t>
+          <t>HTTP 200 com body {"message": "Webhook processado"}</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -4044,7 +4044,7 @@
       <c r="L76" s="2" t="inlineStr"/>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>Cenário Negativo</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -4056,32 +4056,32 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Lista e Detalhe de Psicólogos</t>
+          <t>Assinatura Premium (RevenueCat)</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Verificar filtro de psicólogos por área de interesse do paciente</t>
+          <t>Verificar rejeição de webhook não autorizado</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado com areaInteresse definida.</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Nenhum (GET, token de paciente com areaInteresse)</t>
+          <t>Header Authorization=&lt;secret_errado&gt;</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente com areaInteresse. 2. Enviar GET /api/psicologos com o token. 3. Verificar que a lista é filtrada por correspondência de tags.</t>
+          <t>1. Enviar POST /api/assinatura/webhook com header Authorization incorreto. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 — apenas psicólogos cujo tipoPsicologo corresponde à areaInteresse do paciente (normalização de tags)</t>
+          <t>HTTP 401 com body {"error": "Webhook nao autorizado"}</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -4091,7 +4091,7 @@
       <c r="L77" s="2" t="inlineStr"/>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo — filtro por interesse</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -4103,32 +4103,32 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Lista e Detalhe de Psicólogos</t>
+          <t>Assinatura Premium (RevenueCat)</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Verificar financeiro do psicólogo</t>
+          <t>Verificar rejeição de webhook com payload inválido</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Psicólogo autenticado (JWT).</t>
+          <t>REVENUECAT_WEBHOOK_SECRET configurado no backend.</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>periodo='mes'</t>
+          <t>Header Authorization=&lt;secret&gt;. Body: {"event": {}}</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do psicólogo demo. 2. Enviar GET /api/psicologos/financeiro?periodo=mes. 3. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar POST /api/assinatura/webhook com payload sem type/app_user_id. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com faturamentoMes, consultasRealizadas, ticketMedio e transacoes (últimas 20 não-canceladas)</t>
+          <t>HTTP 400 com body {"error": "Payload RevenueCat invalido"}</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -4138,7 +4138,7 @@
       <c r="L78" s="2" t="inlineStr"/>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Campo obrigatório vazio</t>
         </is>
       </c>
     </row>
@@ -4150,32 +4150,32 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Lista e Detalhe de Psicólogos</t>
+          <t>Assinatura Premium (RevenueCat)</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de acesso ao financeiro sem token JWT</t>
+          <t>Verificar status de assinatura de usuário free</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente autenticado sem assinatura ativa.</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>periodo='mes' (sem token)</t>
+          <t>Nenhum (GET)</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar GET /api/psicologos/financeiro sem header Authorization. 2. Verificar o código HTTP.</t>
+          <t>1. Obter token JWT do paciente demo (não-premium). 2. Enviar GET /api/assinatura/status com o token. 3. Verificar o corpo da resposta.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>HTTP 401 (endpoint exige JWT)</t>
+          <t>HTTP 200 com body {"isPremium": false, "chamadasRealizadas": &lt;count&gt;, "limiteMensal": 4}</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -4185,7 +4185,7 @@
       <c r="L79" s="2" t="inlineStr"/>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Cenário Positivo — limite gratuito de 4 sessões/mês</t>
         </is>
       </c>
     </row>
@@ -4197,32 +4197,32 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Chat em Tempo Real (WebSocket STOMP)</t>
+          <t>Assinatura Premium (RevenueCat)</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Verificar conexão WebSocket com token JWT válido</t>
+          <t>Verificar status de assinatura sem token JWT</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Paciente autenticado (JWT válido).</t>
+          <t>Sistema no ar.</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>ws://&lt;host&gt;/ws-chat?token=&lt;jwt_válido&gt;</t>
+          <t>Nenhum (GET, sem token)</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>1. Obter token JWT do paciente demo. 2. Conectar ao endpoint /ws-chat?token=&lt;token&gt;. 3. Verificar se a conexão é estabelecida (CONNECTED).</t>
+          <t>1. Enviar GET /api/assinatura/status sem header Authorization. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Conexão estabelecida com sucesso (frame CONNECTED do STOMP)</t>
+          <t>HTTP 401 (endpoint exige JWT)</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -4232,7 +4232,7 @@
       <c r="L80" s="2" t="inlineStr"/>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -4244,32 +4244,32 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Chat em Tempo Real (WebSocket STOMP)</t>
+          <t>Gestão de Usuários (Admin)</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de conexão WebSocket com token inválido</t>
+          <t>Verificar listagem de todos os usuários por admin</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Admin autenticado (JWT).</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>ws://&lt;host&gt;/ws-chat?token=token_invalido</t>
+          <t>Nenhum (GET)</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>1. Conectar ao endpoint /ws-chat com token inválido. 2. Verificar se a conexão é recusada.</t>
+          <t>1. Obter token JWT do admin (admin@cedro.com). 2. Enviar GET /api/usuarios com o token. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Conexão recusada (handshake falha — StompHandshakeInterceptor valida token na query string)</t>
+          <t>HTTP 200 com lista de todos os usuários</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -4279,7 +4279,7 @@
       <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Cenário Positivo — NOTA: endpoint expõe senhaHash (vulnerabilidade conhecida)</t>
         </is>
       </c>
     </row>
@@ -4291,32 +4291,32 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Chat em Tempo Real (WebSocket STOMP)</t>
+          <t>Gestão de Usuários (Admin)</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de conexão WebSocket com token expirado</t>
+          <t>Verificar rejeição de listagem de usuários por não-admin</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Token JWT expirado (24h de validade).</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>ws://&lt;host&gt;/ws-chat?token=&lt;jwt_expirado&gt;</t>
+          <t>Nenhum (GET, token de paciente)</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>1. Gerar token JWT expirado. 2. Conectar ao endpoint /ws-chat com token expirado. 3. Verificar se a conexão é recusada.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar GET /api/usuarios com o token do paciente. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Conexão recusada (token expirado)</t>
+          <t>HTTP 403 com body {"error": "Acesso negado"}</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -4338,32 +4338,32 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Chat em Tempo Real (WebSocket STOMP)</t>
+          <t>Gestão de Usuários (Admin)</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Verificar envio e recebimento de mensagem via STOMP</t>
+          <t>Verificar que usuário comum só pode ver a si mesmo</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Paciente e psicólogo conectados ao WebSocket com tokens válidos.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>destination='/app/chat.send', body={"destinatarioId": &lt;id_psicologo&gt;, "mensagem": "Olá via STOMP"}</t>
+          <t>id=&lt;id_de_outro_usuario&gt; (token do paciente)</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>1. Conectar paciente e psicólogo ao WebSocket. 2. Paciente publica em /app/chat.send. 3. Verificar que o psicólogo recebe em /user/queue/mensagens.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar GET /api/usuarios/{id} de outro usuário. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Psicólogo recebe payload {"type": "chat:message", "mensagem": &lt;Mensagem&gt;}</t>
+          <t>HTTP 403 (se não admin e id não corresponde)</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -4373,7 +4373,7 @@
       <c r="L83" s="2" t="inlineStr"/>
       <c r="M83" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo — chat em tempo real</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -4385,32 +4385,32 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Chat em Tempo Real (WebSocket STOMP)</t>
+          <t>Gestão de Usuários (Admin)</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Verificar conexão WebSocket sem token</t>
+          <t>Verificar ativação/desativação de usuário por admin</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Admin autenticado (JWT).</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>ws://&lt;host&gt;/ws-chat (sem parâmetro token)</t>
+          <t>id=&lt;id_usuario&gt;, body={"ativo": false}</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>1. Conectar ao endpoint /ws-chat sem token na query string. 2. Verificar se a conexão é recusada.</t>
+          <t>1. Obter token JWT do admin. 2. Enviar PUT /api/usuarios/{id}/ativar com ativo=false. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Conexão recusada (token ausente)</t>
+          <t>HTTP 200 com body {"message": "ok"}</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -4420,7 +4420,7 @@
       <c r="L84" s="2" t="inlineStr"/>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>Acesso não autorizado</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -4432,32 +4432,32 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Recuperação e Redefinição de Senha</t>
+          <t>Gestão de Usuários (Admin)</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Verificar solicitação de recuperação de senha</t>
+          <t>Verificar rejeição de desativação de usuário por não-admin</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Paciente autenticado (JWT).</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>email='paciente.demo@cedro.app'</t>
+          <t>id=&lt;id_usuario&gt;, body={"ativo": false} (token de paciente)</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/auth/recuperar-senha com email do paciente demo. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar PUT /api/usuarios/{id}/ativar com o token do paciente. 3. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"message": "Se o e-mail existir, enviaremos instrucoes"}</t>
+          <t>HTTP 403 (apenas admin)</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -4467,7 +4467,7 @@
       <c r="L85" s="2" t="inlineStr"/>
       <c r="M85" s="2" t="inlineStr">
         <is>
-          <t>Cenário Positivo — mensagem genérica (não revela se email existe)</t>
+          <t>Acesso não autorizado</t>
         </is>
       </c>
     </row>
@@ -4479,32 +4479,32 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Recuperação e Redefinição de Senha</t>
+          <t>Gestão de Usuários (Admin)</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Verificar solicitação de recuperação com email inexistente</t>
+          <t>Verificar exclusão de usuário por admin</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Admin autenticado (JWT). Usuário de teste criado.</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>email='naoexiste.22241168@teste.cedro'</t>
+          <t>id=&lt;id_usuario_teste&gt;</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/auth/recuperar-senha com email não cadastrado. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do admin. 2. Enviar DELETE /api/usuarios/{id} do usuário de teste. 3. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 com body {"message": "Se o e-mail existir, enviaremos instrucoes"} (mesma mensagem — não revela se email existe)</t>
+          <t>HTTP 200 com body {"message": "Deletada"}</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -4514,7 +4514,7 @@
       <c r="L86" s="2" t="inlineStr"/>
       <c r="M86" s="2" t="inlineStr">
         <is>
-          <t>Cenário Negativo — segurança por obscuridade</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -4526,32 +4526,32 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Recuperação e Redefinição de Senha</t>
+          <t>Lista e Detalhe de Psicólogos</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de recuperação com email vazio</t>
+          <t>Verificar listagem pública de psicólogos</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Sistema no ar. Psicólogos cadastrados.</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>email=''</t>
+          <t>Nenhum (GET, público)</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/auth/recuperar-senha com email vazio. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar GET /api/psicologos sem autenticação. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Informe o email"}</t>
+          <t>HTTP 200 com lista de DTOs públicos {id, nome, especialidade, tipoPsicologo, bio, precoSessao, avaliacao, fotoUrl} — sem email, telefone ou senha</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -4561,7 +4561,7 @@
       <c r="L87" s="2" t="inlineStr"/>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>Campo obrigatório vazio</t>
+          <t>Cenário Positivo</t>
         </is>
       </c>
     </row>
@@ -4573,12 +4573,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Recuperação e Redefinição de Senha</t>
+          <t>Lista e Detalhe de Psicólogos</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Verificar redefinição de senha com token inválido</t>
+          <t>Verificar detalhe de psicólogo inexistente</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -4588,17 +4588,17 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>token='token_invalido', novaSenha='NovaSenha@123'</t>
+          <t>id=999999</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/auth/redefinir-senha com token inválido. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar GET /api/psicologos/999999. 2. Verificar o código HTTP.</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Token invalido ou expirado"}</t>
+          <t>HTTP 400 (RuntimeException 'Não encontrado' tratada pelo GlobalExceptionHandler)</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr"/>
@@ -4620,32 +4620,32 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Recuperação e Redefinição de Senha</t>
+          <t>Lista e Detalhe de Psicólogos</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de redefinição sem token</t>
+          <t>Verificar detalhe de usuário que não é psicólogo</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Sistema no ar.</t>
+          <t>Sistema no ar. Paciente demo cadastrado.</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>novaSenha='NovaSenha@123' (sem token)</t>
+          <t>id=&lt;id_paciente_demo&gt;</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/auth/redefinir-senha sem o campo token. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Enviar GET /api/psicologos/{id} do paciente demo. 2. Verificar o código HTTP e o corpo da resposta.</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Token e nova senha sao obrigatorios"}</t>
+          <t>HTTP 400 com body {"error": "Não é psicólogo"}</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr"/>
@@ -4655,7 +4655,7 @@
       <c r="L89" s="2" t="inlineStr"/>
       <c r="M89" s="2" t="inlineStr">
         <is>
-          <t>Campo obrigatório vazio</t>
+          <t>Cenário Negativo</t>
         </is>
       </c>
     </row>
@@ -4667,32 +4667,32 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Recuperação e Redefinição de Senha</t>
+          <t>Lista e Detalhe de Psicólogos</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Verificar rejeição de redefinição com token expirado</t>
+          <t>Verificar filtro de psicólogos por área de interesse do paciente</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Token de redefinição expirado (30 minutos de validade).</t>
+          <t>Paciente autenticado com areaInteresse definida.</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>token='&lt;token_expirado&gt;', novaSenha='NovaSenha@123'</t>
+          <t>Nenhum (GET, token de paciente com areaInteresse)</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>1. Enviar POST /api/auth/redefinir-senha com token expirado. 2. Verificar o código HTTP e o corpo da resposta.</t>
+          <t>1. Obter token JWT do paciente com areaInteresse. 2. Enviar GET /api/psicologos com o token. 3. Verificar que a lista é filtrada por correspondência de tags.</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400 com body {"error": "Token invalido ou expirado"}</t>
+          <t>HTTP 200 — apenas psicólogos cujo tipoPsicologo corresponde à areaInteresse do paciente (normalização de tags)</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr"/>
@@ -4702,27 +4702,967 @@
       <c r="L90" s="2" t="inlineStr"/>
       <c r="M90" s="2" t="inlineStr">
         <is>
+          <t>Cenário Positivo — filtro por interesse</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>CT-091</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Lista e Detalhe de Psicólogos</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Verificar financeiro do psicólogo</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Psicólogo autenticado (JWT).</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>periodo='mes'</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>1. Obter token JWT do psicólogo demo. 2. Enviar GET /api/psicologos/financeiro?periodo=mes. 3. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200 com faturamentoMes, consultasRealizadas, ticketMedio e transacoes (últimas 20 não-canceladas)</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr"/>
+      <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="inlineStr"/>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>Cenário Positivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>CT-092</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Lista e Detalhe de Psicólogos</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Verificar rejeição de acesso ao financeiro sem token JWT</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Sistema no ar.</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>periodo='mes' (sem token)</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>1. Enviar GET /api/psicologos/financeiro sem header Authorization. 2. Verificar o código HTTP.</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 401 (endpoint exige JWT)</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr"/>
+      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr"/>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>Acesso não autorizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>CT-093</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard Psicólogo</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Verificar estatísticas do psicólogo autenticado</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Psicólogo autenticado (JWT).</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>Nenhum (GET)</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>1. Obter token JWT do psicólogo demo. 2. Enviar GET /api/psicologos/estatisticas com o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200 com body {consultasHoje, consultasSemana, pacientesAtivos, faturamentoMes}</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr"/>
+      <c r="I93" s="2" t="inlineStr"/>
+      <c r="J93" s="2" t="inlineStr"/>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="2" t="inlineStr"/>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>Cenário Positivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>CT-094</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard Psicólogo</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Verificar próximas consultas do psicólogo</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Psicólogo autenticado (JWT).</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Nenhum (GET)</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>1. Obter token JWT do psicólogo demo. 2. Enviar GET /api/psicologos/consultas/proximas com o token. 3. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200 com lista de até 10 sessões futuras ordenadas por data asc, cada item com {id, pacienteId, data, horario, status, tipo, pacienteNome}</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr"/>
+      <c r="I94" s="2" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr"/>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>Cenário Positivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>CT-095</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard Psicólogo</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Verificar rejeição de acesso às estatísticas sem token JWT</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Sistema no ar.</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>Nenhum (GET, sem token)</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>1. Enviar GET /api/psicologos/estatisticas sem header Authorization. 2. Verificar o código HTTP.</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 401 (endpoint exige JWT)</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr"/>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>Acesso não autorizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>CT-096</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Chat em Tempo Real (WebSocket STOMP)</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Verificar conexão WebSocket com token JWT válido</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Paciente autenticado (JWT válido).</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>ws://&lt;host&gt;/ws-chat?token=&lt;jwt_válido&gt;</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>1. Obter token JWT do paciente demo. 2. Conectar ao endpoint /ws-chat?token=&lt;token&gt;. 3. Verificar se a conexão é estabelecida (CONNECTED).</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Conexão estabelecida com sucesso (frame CONNECTED do STOMP)</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr"/>
+      <c r="I96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>Cenário Positivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>CT-097</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Chat em Tempo Real (WebSocket STOMP)</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Verificar rejeição de conexão WebSocket com token inválido</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Sistema no ar.</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>ws://&lt;host&gt;/ws-chat?token=token_invalido</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>1. Conectar ao endpoint /ws-chat com token inválido. 2. Verificar se a conexão é recusada.</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Conexão recusada (handshake falha — StompHandshakeInterceptor valida token na query string)</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr"/>
+      <c r="I97" s="2" t="inlineStr"/>
+      <c r="J97" s="2" t="inlineStr"/>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr"/>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>Acesso não autorizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>CT-098</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Chat em Tempo Real (WebSocket STOMP)</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Verificar rejeição de conexão WebSocket com token expirado</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Token JWT expirado (24h de validade).</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>ws://&lt;host&gt;/ws-chat?token=&lt;jwt_expirado&gt;</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>1. Gerar token JWT expirado. 2. Conectar ao endpoint /ws-chat com token expirado. 3. Verificar se a conexão é recusada.</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Conexão recusada (token expirado)</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>Acesso não autorizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>CT-099</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Chat em Tempo Real (WebSocket STOMP)</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Verificar envio e recebimento de mensagem via STOMP</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Paciente e psicólogo conectados ao WebSocket com tokens válidos.</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>destination='/app/chat.send', body={"destinatarioId": &lt;id_psicologo&gt;, "mensagem": "Olá via STOMP"}</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>1. Conectar paciente e psicólogo ao WebSocket. 2. Paciente publica em /app/chat.send. 3. Verificar que o psicólogo recebe em /user/queue/mensagens.</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Psicólogo recebe payload {"type": "chat:message", "mensagem": &lt;Mensagem&gt;}</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr"/>
+      <c r="I99" s="2" t="inlineStr"/>
+      <c r="J99" s="2" t="inlineStr"/>
+      <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr"/>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>Cenário Positivo — chat em tempo real</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>CT-100</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Chat em Tempo Real (WebSocket STOMP)</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Verificar conexão WebSocket sem token</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Sistema no ar.</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>ws://&lt;host&gt;/ws-chat (sem parâmetro token)</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>1. Conectar ao endpoint /ws-chat sem token na query string. 2. Verificar se a conexão é recusada.</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Conexão recusada (token ausente)</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr"/>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr"/>
+      <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr"/>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>Acesso não autorizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>CT-101</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Recuperação e Redefinição de Senha</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Verificar solicitação de recuperação de senha</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Sistema no ar.</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>email='paciente.demo@cedro.app'</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>1. Enviar POST /api/auth/recuperar-senha com email do paciente demo. 2. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200 com body {"message": "Se o e-mail existir, enviaremos instrucoes"}</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr"/>
+      <c r="I101" s="2" t="inlineStr"/>
+      <c r="J101" s="2" t="inlineStr"/>
+      <c r="K101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr"/>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>Cenário Positivo — mensagem genérica (não revela se email existe)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>CT-102</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Recuperação e Redefinição de Senha</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Verificar solicitação de recuperação com email inexistente</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Sistema no ar.</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>email='naoexiste.35f5031a@teste.cedro'</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>1. Enviar POST /api/auth/recuperar-senha com email não cadastrado. 2. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200 com body {"message": "Se o e-mail existir, enviaremos instrucoes"} (mesma mensagem — não revela se email existe)</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr"/>
+      <c r="I102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr"/>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr"/>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>Cenário Negativo — segurança por obscuridade</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>CT-103</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Recuperação e Redefinição de Senha</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Verificar rejeição de recuperação com email vazio</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Sistema no ar.</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>email=''</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>1. Enviar POST /api/auth/recuperar-senha com email vazio. 2. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400 com body {"error": "Informe o email"}</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr"/>
+      <c r="I103" s="2" t="inlineStr"/>
+      <c r="J103" s="2" t="inlineStr"/>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="2" t="inlineStr"/>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>Campo obrigatório vazio</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>CT-104</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Recuperação e Redefinição de Senha</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Verificar redefinição de senha com token inválido</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Sistema no ar.</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>token='token_invalido', novaSenha='NovaSenha@123'</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>1. Enviar POST /api/auth/redefinir-senha com token inválido. 2. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400 com body {"error": "Token invalido ou expirado"}</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="inlineStr"/>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>Cenário Negativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>CT-105</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Recuperação e Redefinição de Senha</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Verificar rejeição de redefinição sem token</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Sistema no ar.</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>novaSenha='NovaSenha@123' (sem token)</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>1. Enviar POST /api/auth/redefinir-senha sem o campo token. 2. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400 com body {"error": "Token e nova senha sao obrigatorios"}</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr"/>
+      <c r="I105" s="2" t="inlineStr"/>
+      <c r="J105" s="2" t="inlineStr"/>
+      <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="2" t="inlineStr"/>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>Campo obrigatório vazio</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>CT-106</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Recuperação e Redefinição de Senha</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Verificar rejeição de redefinição com token expirado</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Token de redefinição expirado (30 minutos de validade).</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>token='&lt;token_expirado&gt;', novaSenha='NovaSenha@123'</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>1. Enviar POST /api/auth/redefinir-senha com token expirado. 2. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400 com body {"error": "Token invalido ou expirado"}</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr"/>
+      <c r="I106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr"/>
+      <c r="K106" s="2" t="inlineStr"/>
+      <c r="L106" s="2" t="inlineStr"/>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
           <t>Valor no limite — expiração de 30 minutos</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="2" t="n"/>
-      <c r="B91" s="2" t="n"/>
-      <c r="C91" s="2" t="n"/>
-      <c r="D91" s="2" t="n"/>
-      <c r="E91" s="2" t="n"/>
-      <c r="F91" s="2" t="n"/>
-      <c r="G91" s="2" t="n"/>
-      <c r="H91" s="2" t="n"/>
-      <c r="I91" s="2" t="n"/>
-      <c r="J91" s="2" t="n"/>
-      <c r="K91" s="2" t="n"/>
-      <c r="L91" s="2" t="n"/>
-      <c r="M91" s="2" t="n"/>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>CT-107</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Notificações Push</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Verificar registro de push token válido</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>Paciente autenticado (JWT).</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>token='ExponentPushToken[xxxxxxxxxxxxxxxxxxxxxx]'</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/notificacoes/token com body {token: '...'}. 3. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200 com body {"message": "Token registrado"}</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr"/>
+      <c r="I107" s="2" t="inlineStr"/>
+      <c r="J107" s="2" t="inlineStr"/>
+      <c r="K107" s="2" t="inlineStr"/>
+      <c r="L107" s="2" t="inlineStr"/>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>Cenário Positivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>CT-108</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Notificações Push</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Verificar remoção de push token</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Paciente autenticado (JWT). Token previamente registrado.</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>token='ExponentPushToken[xxxxxxxxxxxxxxxxxxxxxx]'</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/notificacoes/token/remover com body {token: '...'}. 3. Verificar o código HTTP e o corpo da resposta.</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200 com body {"message": "Token removido"}</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr"/>
+      <c r="I108" s="2" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr"/>
+      <c r="K108" s="2" t="inlineStr"/>
+      <c r="L108" s="2" t="inlineStr"/>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>Cenário Positivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>CT-109</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Notificações Push</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Verificar rejeição de registro de token sem autenticação</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Sistema no ar.</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>token='ExponentPushToken[xxxxxxxxxxxxxxxxxxxxxx]' (sem token JWT)</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>1. Enviar POST /api/notificacoes/token sem header Authorization. 2. Verificar o código HTTP.</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 401 (endpoint exige JWT)</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr"/>
+      <c r="I109" s="2" t="inlineStr"/>
+      <c r="J109" s="2" t="inlineStr"/>
+      <c r="K109" s="2" t="inlineStr"/>
+      <c r="L109" s="2" t="inlineStr"/>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>Acesso não autorizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>CT-110</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Notificações Push</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Verificar que token duplicado não gera erro (idempotente)</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Paciente autenticado (JWT). Token já registrado.</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>token='ExponentPushToken[xxxxxxxxxxxxxxxxxxxxxx]' (mesmo token)</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>1. Obter token JWT do paciente demo. 2. Enviar POST /api/notificacoes/token com o mesmo token duas vezes. 3. Verificar o código HTTP na segunda chamada.</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 200 — o service verifica duplicidade antes de inserir (índice único UX_push_tokens_usuario_token)</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr"/>
+      <c r="I110" s="2" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr"/>
+      <c r="K110" s="2" t="inlineStr"/>
+      <c r="L110" s="2" t="inlineStr"/>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>Registro duplicado — comportamento idempotente</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n"/>
+      <c r="B111" s="2" t="n"/>
+      <c r="C111" s="2" t="n"/>
+      <c r="D111" s="2" t="n"/>
+      <c r="E111" s="2" t="n"/>
+      <c r="F111" s="2" t="n"/>
+      <c r="G111" s="2" t="n"/>
+      <c r="H111" s="2" t="n"/>
+      <c r="I111" s="2" t="n"/>
+      <c r="J111" s="2" t="n"/>
+      <c r="K111" s="2" t="n"/>
+      <c r="L111" s="2" t="n"/>
+      <c r="M111" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M91"/>
+  <autoFilter ref="A1:M111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>